<commit_message>
Schedule: bring M5-M7 topics in line with notes v4.1; add handout column
M5B adds isotonic recalibration and the paired comparison of two policies; M6A adds group
constraints (price of fairness) and capacity (critical fractile); M6B replaces 'plug-in vs
direct learning' with the predict-then-optimise / decision-focused / policy-learning spectrum;
M7B adds the outcome-free design stage. New column G lists each meeting's handout (H1-H6).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DLgfSPmYNxNjqrXY4qwk61
</commit_message>
<xml_diff>
--- a/plan/schedule.xlsx
+++ b/plan/schedule.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -506,6 +506,7 @@
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -546,6 +547,11 @@
           <t>Bonus reading</t>
         </is>
       </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Handout (not examined)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -572,6 +578,7 @@
           <t>Causal graphs</t>
         </is>
       </c>
+      <c r="G4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
@@ -602,6 +609,11 @@
           <t>Spillover</t>
         </is>
       </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>H4 Interference and marketplace experiments</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -632,6 +644,11 @@
           <t>More deep causal models</t>
         </is>
       </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>H6 Neural and foundation-model estimators</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -662,6 +679,7 @@
           <t>Forest theory</t>
         </is>
       </c>
+      <c r="G7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -674,7 +692,7 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>CATE V: evaluation. Ranking vs calibration; uplift and Qini curves; RATE; policy value on held-out RCT data; the policy-value identity; selection vs evaluation data; freezing a policy</t>
+          <t>CATE V: evaluation. Ranking vs calibration, and isotonic recalibration; uplift and Qini curves; RATE; policy value on held-out RCT data; the policy-value identity; selection vs evaluation data; freezing a policy; comparing two policies (paired SE)</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -692,6 +710,7 @@
           <t>Evaluating prioritisation rules</t>
         </is>
       </c>
+      <c r="G8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
@@ -699,12 +718,12 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>CATE VI: allocation. Net value per customer; break-even thresholds; budget as a knapsack and its shadow price; customer-specific costs; contact caps; several coupon depths; noisy estimates and lower-bound allocation</t>
+          <t>CATE VI: allocation. Net value per customer; break-even thresholds; budget as a knapsack and its shadow price; customer-specific costs; contact caps; several coupon depths; noisy estimates and lower-bound allocation; group constraints and the price of fairness; capacity and the critical fractile</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>CATE VII: policy learning. Plug-in vs direct learning; DR scores; empirical welfare maximisation; policy trees; regret and policy-class complexity; deploying with holdouts; bandits as continuous experimentation</t>
+          <t>CATE VII: policy learning. Predict-then-optimise, decision-focused learning and policy learning as one spectrum; policy learning as weighted classification with DR scores; empirical welfare maximisation; policy trees; regret and policy-class complexity; deploying with holdouts; bandits as continuous experimentation</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -716,6 +735,11 @@
       <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Policy learning theory; dynamic regimes</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>H5 Sequential decisions</t>
         </is>
       </c>
     </row>
@@ -730,7 +754,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Observational data II: propensity scores. Balancing property; matching and IPW; doubly robust AIPW; overlap diagnostics, trimming and the changed estimand; the LaLonde benchmark; a first look at sensitivity to hidden confounding</t>
+          <t>Observational data II: propensity scores. Balancing property; matching and IPW; doubly robust AIPW; overlap diagnostics, trimming and the changed estimand; the outcome-free design stage; the LaLonde benchmark; a first look at sensitivity to hidden confounding</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -742,6 +766,11 @@
       <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Instrumental variables</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>H1 Instrumental variables</t>
         </is>
       </c>
     </row>
@@ -774,6 +803,11 @@
           <t>Regression discontinuity</t>
         </is>
       </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>H2 Regression discontinuity</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -804,6 +838,7 @@
           <t>Causal transformer</t>
         </is>
       </c>
+      <c r="G12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
@@ -834,6 +869,11 @@
           <t>Staggered DiD</t>
         </is>
       </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>H3 Staggered adoption</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -864,6 +904,7 @@
           <t>Synthetic DiD; matrix completion</t>
         </is>
       </c>
+      <c r="G14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -882,11 +923,12 @@
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr"/>
+      <c r="G15" s="8" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:F15"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Schedule, syllabus, brief: IV core closes M2; A3 due Friday W5; critique exercises dropped
Instructor decisions of 8 Oct. Noncompliance, ITT and the LATE end Experiments II (M2) and
Handout H1 moves with them; M7's bonus slot gets Rubin (2008) and Crump et al. (2009). A3
moves to Friday of Week 5 so nothing is due the weekend before Exam II. Reading-and-critique
exercises are removed from the syllabus and the brief. The brief records which judgement
calls are now decided and the one opened by the IV move (M2 notes and H1 location).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DLgfSPmYNxNjqrXY4qwk61
</commit_message>
<xml_diff>
--- a/plan/schedule.xlsx
+++ b/plan/schedule.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Experiments II: design. Power and MDE for a decision; randomisation unit and clustered SEs; interference; peeking and multiple metrics; noncompliance (ITT vs effect of redemption); transport to a new campaign</t>
+          <t>Experiments II: design. Power and MDE for a decision; randomisation unit and clustered SEs; interference; peeking and multiple metrics; transport to a new campaign; to close, noncompliance and instruments: ITT and first stage, compliance types, the LATE and its assumptions, the Wald ratio</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>H4 Interference and marketplace experiments</t>
+          <t>H4 Interference and marketplace experiments; H1 Instrumental variables</t>
         </is>
       </c>
     </row>
@@ -768,11 +768,7 @@
           <t>Instrumental variables</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>H1 Instrumental variables</t>
-        </is>
-      </c>
+      <c r="G10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -861,7 +857,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>A3 due (Sun). Revised identification plan (Sat)</t>
+          <t>A3 due (Fri). Revised identification plan (Sat)</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1416,7 +1412,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Sun W5</t>
+          <t>Fri W5</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1606,7 +1602,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>A3 (Sun)</t>
+          <t>A3 (Fri)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1745,12 +1741,12 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Spillover</t>
+          <t>Spillover; instrumental variables</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Hudgens and Halloran (2008); Johari et al. (2022) on two-sided marketplace experiments; Bojinov, Simchi-Levi and Zhao (2023) on switchbacks; Kohavi, Tang and Xu (2020) as the practitioner reference</t>
+          <t>Hudgens and Halloran (2008); Johari et al. (2022) on two-sided marketplace experiments; Bojinov, Simchi-Levi and Zhao (2023) on switchbacks; Kohavi, Tang and Xu (2020) as the practitioner reference; Angrist, Imbens and Rubin (1996); Angrist and Pischke, Mastering 'Metrics, chapter 3</t>
         </is>
       </c>
     </row>
@@ -1830,12 +1826,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Instrumental variables</t>
+          <t>Design before analysis; limited overlap</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Angrist, Imbens and Rubin (1996); Angrist and Pischke, Mastering 'Metrics, chapter 3</t>
+          <t>Rubin (2008), "For objective causal inference, design trumps analysis"; Crump, Hotz, Imbens and Mitnik (2009), "Dealing with limited overlap"</t>
         </is>
       </c>
     </row>
@@ -1979,12 +1975,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Noncompliance slide</t>
+          <t>Noncompliance and IV in M2</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>IV is bonus-only, but one slide on noncompliance stays in Experiments II (ITT vs effect of redemption), pointing to the bonus reading.</t>
+          <t>Decided (8 Oct): IV, noncompliance and the LATE close Experiments II (M2), in the coffee-chain case; Handout H1 goes with M2 and goes further (2SLS, weak instruments, exclusion failures).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Planning docs: noncompliance in an RCT closes M2; classical IV and H1 stay with M7 as bonus
Corrects the previous commit, which moved all of IV and Handout H1 to M2. Only the ITT and
LATE under noncompliance in an RCT (potential outcomes, the draw as instrument) move to M2;
classical IV stays in H1 with M7 as bonus reading. Spreadsheet, syllabus, brief and README
updated to match; the resolved open call is removed from the brief.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DLgfSPmYNxNjqrXY4qwk61
</commit_message>
<xml_diff>
--- a/plan/schedule.xlsx
+++ b/plan/schedule.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Experiments II: design. Power and MDE for a decision; randomisation unit and clustered SEs; interference; peeking and multiple metrics; transport to a new campaign; to close, noncompliance and instruments: ITT and first stage, compliance types, the LATE and its assumptions, the Wald ratio</t>
+          <t>Experiments II: design. Power and MDE for a decision; randomisation unit and clustered SEs; interference; peeking and multiple metrics; transport to a new campaign; to close, noncompliance in an RCT: ITT and first stage, compliance types, the LATE (potential outcomes; the draw as the instrument)</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>H4 Interference and marketplace experiments; H1 Instrumental variables</t>
+          <t>H4 Interference and marketplace experiments</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,11 @@
           <t>Instrumental variables</t>
         </is>
       </c>
-      <c r="G10" s="4" t="n"/>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>H1 Instrumental variables</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -1741,12 +1745,12 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Spillover; instrumental variables</t>
+          <t>Spillover; noncompliance and the LATE</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Hudgens and Halloran (2008); Johari et al. (2022) on two-sided marketplace experiments; Bojinov, Simchi-Levi and Zhao (2023) on switchbacks; Kohavi, Tang and Xu (2020) as the practitioner reference; Angrist, Imbens and Rubin (1996); Angrist and Pischke, Mastering 'Metrics, chapter 3</t>
+          <t>Hudgens and Halloran (2008); Johari et al. (2022) on two-sided marketplace experiments; Bojinov, Simchi-Levi and Zhao (2023) on switchbacks; Kohavi, Tang and Xu (2020) as the practitioner reference; Angrist, Imbens and Rubin (1996) on the LATE</t>
         </is>
       </c>
     </row>
@@ -1826,12 +1830,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Design before analysis; limited overlap</t>
+          <t>Instrumental variables</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Rubin (2008), "For objective causal inference, design trumps analysis"; Crump, Hotz, Imbens and Mitnik (2009), "Dealing with limited overlap"</t>
+          <t>Angrist and Pischke, Mastering 'Metrics, chapter 3; Handout H1</t>
         </is>
       </c>
     </row>
@@ -1975,12 +1979,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Noncompliance and IV in M2</t>
+          <t>Noncompliance in M2; classical IV as bonus</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Decided (8 Oct): IV, noncompliance and the LATE close Experiments II (M2), in the coffee-chain case; Handout H1 goes with M2 and goes further (2SLS, weak instruments, exclusion failures).</t>
+          <t>Decided (8 Oct): ITT and the LATE under noncompliance in an RCT (potential outcomes, the draw as the instrument) close Experiments II (M2) and its notes. Classical IV (outside shifters in observational data, 2SLS, weak instruments) stays in Handout H1 with M7, as bonus reading.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
M2 slides: rebuild on the coffee-chain case, aligned with notes v4.1 including noncompliance
Block A follows notes 1.1-1.5 and block B 1.6-1.9, ending with ITT, compliance types and the
LATE on Case A's Part M2-R6. Results 1.1-1.16 carry the notes' numbers and wording; critique
and map frames removed. The schedule and syllabus M2 rows now follow the notes' order
(transport in A, CUPED in B). New slides02_check.py covers every number (0 mismatches).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DLgfSPmYNxNjqrXY4qwk61
</commit_message>
<xml_diff>
--- a/plan/schedule.xlsx
+++ b/plan/schedule.xlsx
@@ -586,12 +586,12 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Experiments I: estimation. Difference in means as OLS on a dummy; robust SEs; testing against the break-even, not zero; covariate adjustment and CUPED; balance and sample-ratio checks</t>
+          <t>Experiments I: estimation. Analyse as drawn (the ITT); sample-ratio checks; Fisher's test and Neyman's variance; the usual SE is conservative; difference in means as OLS on a dummy with robust SEs; testing against the break-even, and an interval on net value; transport to a new campaign</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Experiments II: design. Power and MDE for a decision; randomisation unit and clustered SEs; interference; peeking and multiple metrics; transport to a new campaign; to close, noncompliance in an RCT: ITT and first stage, compliance types, the LATE (potential outcomes; the draw as the instrument)</t>
+          <t>Experiments II: design. Fixing the plan in writing; power and MDE for a decision; CUPED; randomisation unit, interference and clustered SEs; peeking and multiple metrics; to close, noncompliance in an RCT: ITT and first stage, compliance types, the LATE (potential outcomes; the draw as the instrument)</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Schedule: split Misc into Release and Due; syllabus weekly table gains Out / due
The spreadsheet's Misc column becomes Release (A1-A4, Lab 7 take-home) and Due (assignments,
proposal, project milestones), and its handout column uses the new numbers. The syllabus's
weekly table moves the handout into the Block C cell and adds an Out / due column; its handout
table is sorted H1-H6. CHANGELOG records both changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DLgfSPmYNxNjqrXY4qwk61
</commit_message>
<xml_diff>
--- a/plan/schedule.xlsx
+++ b/plan/schedule.xlsx
@@ -497,16 +497,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -516,6 +517,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -539,15 +541,20 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>Due</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>Bonus reading</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Handout (not examined)</t>
         </is>
@@ -572,13 +579,14 @@
           <t>Lab 0: Python, probability and statistics review</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr"/>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Causal graphs</t>
         </is>
       </c>
-      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
@@ -601,17 +609,22 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>A1 out. Pairs formed</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
+          <t>Project pairs formed</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
           <t>Spillover</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>H4 Interference and marketplace experiments</t>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>H1 Interference and marketplace experiments</t>
         </is>
       </c>
     </row>
@@ -634,19 +647,20 @@
           <t>Lab 2: meta-learners from scratch</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Question and data idea (Thu)</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>More deep causal models</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>H6 Neural and foundation-model estimators</t>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>H2 Neural and foundation-model estimators</t>
         </is>
       </c>
     </row>
@@ -669,17 +683,18 @@
           <t>Lab 3: causal forest on the coupon RCT</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>A1 due (Fri)</t>
-        </is>
-      </c>
+      <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="inlineStr">
         <is>
+          <t>A1 (Fri)</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
           <t>Forest theory</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -702,15 +717,20 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>A2 out. Proposal due (Sun)</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
+          <t>Proposal (Sun)</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
           <t>Evaluating prioritisation rules</t>
         </is>
       </c>
-      <c r="G8" s="8" t="n"/>
+      <c r="H8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
@@ -731,15 +751,16 @@
           <t>Lab 5: budgeted allocation and policy trees</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>Policy learning theory; dynamic regimes</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>H5 Sequential decisions</t>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>H3 Sequential decisions</t>
         </is>
       </c>
     </row>
@@ -762,15 +783,16 @@
           <t>Lab 6: observational logs built from an RCT, then an agent's analysis audited</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr"/>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Instrumental variables</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>H1 Instrumental variables</t>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>H4 Instrumental variables</t>
         </is>
       </c>
     </row>
@@ -795,17 +817,22 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Lab 7: DML (take-home). A2 due (Sun). A3 out</t>
+          <t>Lab 7 (DML, take-home); A3</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
+          <t>A2 (Sun)</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
           <t>Regression discontinuity</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>H2 Regression discontinuity</t>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>H5 Regression discontinuity</t>
         </is>
       </c>
     </row>
@@ -830,15 +857,16 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>A4 out</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>Causal transformer</t>
         </is>
       </c>
-      <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
@@ -859,19 +887,20 @@
           <t>Lab 9: evaluating an AI rollout with DiD</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>A3 due (Fri). Revised identification plan (Sat)</t>
-        </is>
-      </c>
+      <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="inlineStr">
         <is>
+          <t>A3 (Fri); revised identification plan (Sat)</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
           <t>Staggered DiD</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>H3 Staggered adoption</t>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>H6 Staggered adoption</t>
         </is>
       </c>
     </row>
@@ -894,17 +923,18 @@
           <t>Lab 10: synthetic control from scratch</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>A4 due (Sun)</t>
-        </is>
-      </c>
+      <c r="E14" s="8" t="n"/>
       <c r="F14" s="8" t="inlineStr">
         <is>
+          <t>A4 (Sun)</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
           <t>Synthetic DiD; matrix completion</t>
         </is>
       </c>
-      <c r="G14" s="8" t="n"/>
+      <c r="H14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -917,18 +947,19 @@
       </c>
       <c r="C15" s="8" t="inlineStr"/>
       <c r="D15" s="8" t="inlineStr"/>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Final slides due the Wednesday before; report due the following Thursday</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr"/>
-      <c r="G15" s="8" t="n"/>
+      <c r="E15" s="8" t="n"/>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Final slides (the Wednesday before); final report (the following Thursday)</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr"/>
+      <c r="H15" s="8" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:F15"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1835,7 +1866,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Angrist and Pischke, Mastering 'Metrics, chapter 3; Handout H1</t>
+          <t>Angrist and Pischke, Mastering 'Metrics, chapter 3; Handout H4</t>
         </is>
       </c>
     </row>
@@ -1984,7 +2015,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Decided (8 Oct): ITT and the LATE under noncompliance in an RCT (potential outcomes, the draw as the instrument) close Experiments II (M2) and its notes. Classical IV (outside shifters in observational data, 2SLS, weak instruments) stays in Handout H1 with M7, as bonus reading.</t>
+          <t>Decided (8 Oct): ITT and the LATE under noncompliance in an RCT (potential outcomes, the draw as the instrument) close Experiments II (M2) and its notes. Classical IV (outside shifters in observational data, 2SLS, weak instruments) stays in Handout H4 with M7, as bonus reading.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Case A, schedule, syllabus: align M4-M6 with the rebuilt decks and the notes
Case A: release table retimed for M4-M6; M4-R3/R4/R5, M5-R1/R4 and M6-R1/R2
updated to the decks' exact numbers (simulated values dropped), keys follow.
Schedule and syllabus rows for M4-M6 reordered to the notes. Brief, README and
changelog record M1-M6 as rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DLgfSPmYNxNjqrXY4qwk61
</commit_message>
<xml_diff>
--- a/plan/schedule.xlsx
+++ b/plan/schedule.xlsx
@@ -670,12 +670,12 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>CATE III: causal forest A. Causal trees that split on effect heterogeneity; honesty and sample splitting; the winner's curse; committing a discovery</t>
+          <t>CATE III: causal trees. An estimand chosen by the data; causal trees that split on effect heterogeneity; the winner's curse; honesty and sample splitting; committing a discovery (discover, estimate, recommend)</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>CATE IV: causal forest B. Forests as adaptive neighbours; local centering (link to the R-learner); CATE intervals and their limits; variable-importance pitfalls; BLP, calibration test, GATES</t>
+          <t>CATE IV: causal forests. Forests as adaptive neighbours; the forest estimate and local centering (link to the R-learner); CATE intervals and their limits; variable-importance pitfalls; BLP calibration test and GATES</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>CATE V: evaluation. Ranking vs calibration, and isotonic recalibration; uplift and Qini curves; RATE; policy value on held-out RCT data; the policy-value identity; selection vs evaluation data; freezing a policy; comparing two policies (paired SE)</t>
+          <t>CATE V: evaluation. Policy value and the policy-value identity; IPW value on held-out RCT data and its variance; gain, profit and Qini curves; RATE; ranking vs calibration, and isotonic recalibration; selection vs evaluation data; freezing a policy; comparing two policies (paired SE)</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -738,12 +738,12 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>CATE VI: allocation. Net value per customer; break-even thresholds; budget as a knapsack and its shadow price; customer-specific costs; contact caps; several coupon depths; noisy estimates and lower-bound allocation; group constraints and the price of fairness; capacity and the critical fractile</t>
+          <t>CATE VI: allocation. Net value per customer and break-even thresholds; customer-specific costs and the sure-thing cost; contact caps; budget as a knapsack and its shadow price; several coupon depths; group constraints and the price of fairness; spending risk and the reserve; noisy estimates and lower-bound allocation; capacity and the critical fractile</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>CATE VII: policy learning. Predict-then-optimise, decision-focused learning and policy learning as one spectrum; policy learning as weighted classification with DR scores; empirical welfare maximisation; policy trees; regret and policy-class complexity; deploying with holdouts; bandits as continuous experimentation</t>
+          <t>CATE VII: policy learning. Predict-then-optimise, decision-focused learning and policy learning as one spectrum; empirical welfare maximisation with DR scores; policy learning as weighted classification; policy trees; regret and policy-class complexity; deploying with holdouts; bandits as continuous experimentation; what the sum assumes (interference, support)</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Schedule, syllabus, brief: align M7-M11 rows with the notes; record all decks rebuilt
Schedule and syllabus rows for M7, M8, M10 and M11 follow the notes' order;
the M9 syllabus row gains its missing simulator topics and a settled case.
The brief, README and changelog record that all eleven decks are rebuilt and
under review, with the decisions still to confirm.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DLgfSPmYNxNjqrXY4qwk61
</commit_message>
<xml_diff>
--- a/plan/schedule.xlsx
+++ b/plan/schedule.xlsx
@@ -770,12 +770,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Observational data I: adjustment. Logs produced by a targeting rule; exchangeability, positivity, consistency; standardisation (g-computation); good and bad controls (mediators, colliders, post-treatment variables); regression adjustment and extrapolation</t>
+          <t>Observational data I: identification and adjustment. Logs produced by a targeting rule; exchangeability, overlap, consistency; standardisation (g-computation) and IPW; the balancing property; what regression adjustment estimates; good and bad controls (mediators, colliders, M-bias, post-treatment variables)</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Observational data II: propensity scores. Balancing property; matching and IPW; doubly robust AIPW; overlap diagnostics, trimming and the changed estimand; the outcome-free design stage; the LaLonde benchmark; a first look at sensitivity to hidden confounding</t>
+          <t>Observational data II: overlap, design and double robustness. Overlap diagnostics, trimming and the changed estimand; the outcome-free design stage; doubly robust AIPW; the LaLonde benchmark; a first look at sensitivity to hidden confounding</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -802,12 +802,12 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>DML I. Why plug-in ML fails (regularisation and overfitting bias); the partially linear model; residualisation (FWL); orthogonality in words; cross-fitting; price elasticity</t>
+          <t>DML I. The partially linear model; residualisation (FWL) and what theta averages when effects vary; why plug-in ML fails (regularisation and overfitting bias); cross-fitting; orthogonality in words; price elasticity</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>DML II. Inference and repeated splits; choice of nuisance learners; the interactive model and AIPW scores; DML for CATE; overlap; omitted-variable sensitivity bounds and benchmarking</t>
+          <t>DML II. Inference and repeated splits; choice of nuisance learners; overlap with a continuous treatment; the interactive model and AIPW scores; DML for CATE; omitted-variable sensitivity bounds and benchmarking</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -874,12 +874,12 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Panel data I: basics. Before-after and its failures (trends, seasonality, regression to the mean); unit and time fixed effects; the within transformation; what fixed effects cannot remove; clustered SEs</t>
+          <t>Panel data I: basics. Adoption-date potential outcomes and the ATT; before-after and its failures (trends, seasonality, regression to the mean); comparisons across units; unit and time fixed effects; the within transformation; what fixed effects cannot remove</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Panel data II: DiD. 2x2 DiD and the ATT; parallel trends (levels vs logs); TWFE with one adoption date; event studies; pre-trend tests and their limits; trend sensitivity; a warning on staggered timing</t>
+          <t>Panel data II: DiD. Parallel trends and no anticipation; 2x2 DiD and the ATT; parallel trends in levels vs logs; TWFE with one adoption date; event studies; pre-trend tests and their limits; trend sensitivity (breakdown drift); inference with one change per unit and clustered SEs; a warning on staggered timing</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Panel data III: synthetic controls. One treated unit; donor weights and pre-period fit; interpolation vs extrapolation; donor pool choice; placebo inference; leave-one-out; limits (poor fit, spillovers, anticipation); SC vs DiD</t>
+          <t>Panel data III: synthetic controls. One treated unit; donor weights and pre-period fit; interpolation vs extrapolation; the factor-model rationale and a long pre-period; design before the post-period; placebo inference in space and in time, and when a rank is a p-value; leave-one-out; limits (extreme units, spillovers, anticipation, local shocks); SC vs DiD</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Calendar, labs, assignments: dated schedule, Labs 1-11 by meeting, new A3/A4 scope
Dates set: Tue/Thu 20 Oct to 1 Dec 2026, no meeting on Thanksgiving (26 Nov).
Labs renumbered to match meetings; ten graded at 1 point each, Lab 7 optional
(its observational methods are graded in A3); no fixed lab deadlines. Proposal
presentations move to M7 and Lab 8 runs in class in M8. A3 covers M7-M9 with a
simulator as the evaluation testbed; A4 is the panel assignment; the hotel
simulator assignment is retired. Final slides and report are due together on
8 Dec. Schedule, syllabus, brief, README and Case A follow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DLgfSPmYNxNjqrXY4qwk61
</commit_message>
<xml_diff>
--- a/plan/schedule.xlsx
+++ b/plan/schedule.xlsx
@@ -15,7 +15,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Judgment calls" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schedule'!$A$3:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Labs'!$A$3:$E$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Assignments'!$A$1:$F$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Deadlines'!$A$3:$D$11</definedName>
@@ -29,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,8 +57,13 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -79,6 +83,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE8D5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E5E7EB"/>
       </patternFill>
     </fill>
   </fills>
@@ -108,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -130,6 +139,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -497,23 +515,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Tuesday/Thursday meetings in Weeks 1 to 5; Thursday in Weeks 6 and 7. Shaded rows contain an exam or the proposals.</t>
+          <t>Tuesdays and Thursdays, 20 October to 1 December 2026; no meeting on Thursday 26 November (Thanksgiving). Shaded rows contain an exam, the proposal presentations or the final presentations. Lab N goes with Meeting N; lab notebooks are expected soon after their meeting and carry no fixed deadline.</t>
         </is>
       </c>
     </row>
@@ -526,35 +545,40 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>A (50 min)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>B (50 min)</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>C (60 min)</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Release</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Bonus reading</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Handout (not examined)</t>
         </is>
@@ -566,27 +590,32 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
+          <t>Tue 20 Oct</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
           <t>Causal basics I: potential outcomes. The decision and its break-even lift; Y(1), Y(0); ATE, ATT, CATE; the fundamental problem; naive difference = ATT + selection bias; SUTVA (no interference, well-defined treatment)</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Causal basics II: causal graphs. DAGs as assumptions; forks, chains, colliders; backdoor paths; randomisation as graph surgery; Simpson's paradox; identification vs estimation vs inference</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Lab 0: Python, probability and statistics review</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="n"/>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Lab 1: Python, probability and statistics review</t>
+        </is>
+      </c>
       <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Causal graphs</t>
         </is>
       </c>
-      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
@@ -594,35 +623,40 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
+          <t>Thu 22 Oct</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
           <t>Experiments I: estimation. Analyse as drawn (the ITT); sample-ratio checks; Fisher's test and Neyman's variance; the usual SE is conservative; difference in means as OLS on a dummy with robust SEs; testing against the break-even, and an interval on net value; transport to a new campaign</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Experiments II: design. Fixing the plan in writing; power and MDE for a decision; CUPED; randomisation unit, interference and clustered SEs; peeking and multiple metrics; to close, noncompliance in an RCT: ITT and first stage, compliance types, the LATE (potential outcomes; the draw as the instrument)</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Lab 1: A/B readout, then an LLM-generated readout checked by simulation tests</t>
-        </is>
-      </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
+          <t>Lab 2: A/B readout, then an LLM-generated readout checked by simulation tests</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Project pairs formed</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Spillover</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>H1 Interference and marketplace experiments</t>
         </is>
@@ -634,31 +668,36 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
+          <t>Tue 27 Oct</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
           <t>CATE I: basics. Why the average misleads targeting; tau(x); effect modifiers vs prognostic variables; persuadables vs sure things; pre-specified subgroups and interaction regressions; multiple testing; GATE (BLP is M4)</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>CATE II: models. S-, T-, X-learners; transformed outcome; DR- and R-learners; TARNet as a shared representation; choosing a model without ground truth (R-loss, DR pseudo-outcomes)</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Lab 2: meta-learners from scratch</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Question and data idea (Thu)</t>
-        </is>
-      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Lab 3: meta-learners from scratch</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="inlineStr">
         <is>
+          <t>Question and data idea (Thu 29 Oct)</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
           <t>More deep causal models</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>H2 Neural and foundation-model estimators</t>
         </is>
@@ -670,31 +709,36 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
+          <t>Thu 29 Oct</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
           <t>CATE III: causal trees. An estimand chosen by the data; causal trees that split on effect heterogeneity; the winner's curse; honesty and sample splitting; committing a discovery (discover, estimate, recommend)</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>CATE IV: causal forests. Forests as adaptive neighbours; the forest estimate and local centering (link to the R-learner); CATE intervals and their limits; variable-importance pitfalls; BLP calibration test and GATES</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Lab 3: causal forest on the coupon RCT</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>A1 (Fri)</t>
-        </is>
-      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Lab 4: causal forest on the coupon RCT</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="inlineStr">
         <is>
+          <t>A1 (Fri 30 Oct)</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
           <t>Forest theory</t>
         </is>
       </c>
-      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -702,35 +746,40 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
+          <t>Tue 3 Nov</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
           <t>EXAM I (M1 to M4)</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>CATE V: evaluation. Policy value and the policy-value identity; IPW value on held-out RCT data and its variance; gain, profit and Qini curves; RATE; ranking vs calibration, and isotonic recalibration; selection vs evaluation data; freezing a policy; comparing two policies (paired SE)</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>Lab 4: four targeting rules evaluated, one of them chosen by an LLM</t>
-        </is>
-      </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
+          <t>Lab 5: CATE evaluation: four targeting rules (one chosen by an LLM) by IPW, Qini and RATE, isotonic recalibration, freeze then evaluate, paired comparison</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Proposal (Sun)</t>
-        </is>
-      </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
+          <t>Proposal (Sun 8 Nov)</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
           <t>Evaluating prioritisation rules</t>
         </is>
       </c>
-      <c r="H8" s="8" t="n"/>
+      <c r="I8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
@@ -738,99 +787,114 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
+          <t>Thu 5 Nov</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
           <t>CATE VI: allocation. Net value per customer and break-even thresholds; customer-specific costs and the sure-thing cost; contact caps; budget as a knapsack and its shadow price; several coupon depths; group constraints and the price of fairness; spending risk and the reserve; noisy estimates and lower-bound allocation; capacity and the critical fractile</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>CATE VII: policy learning. Predict-then-optimise, decision-focused learning and policy learning as one spectrum; empirical welfare maximisation with DR scores; policy learning as weighted classification; policy trees; regret and policy-class complexity; deploying with holdouts; bandits as continuous experimentation; what the sum assumes (interference, support)</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Lab 5: budgeted allocation and policy trees</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="n"/>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Lab 6: budgeted allocation and policy trees</t>
+        </is>
+      </c>
       <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>Policy learning theory; dynamic regimes</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>H3 Sequential decisions</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Tue 10 Nov</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Observational data I: identification and adjustment. Logs produced by a targeting rule; exchangeability, overlap, consistency; standardisation (g-computation) and IPW; the balancing property; what regression adjustment estimates; good and bad controls (mediators, colliders, M-bias, post-treatment variables)</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Observational data II: overlap, design and double robustness. Overlap diagnostics, trimming and the changed estimand; the outcome-free design stage; doubly robust AIPW; the LaLonde benchmark; a first look at sensitivity to hidden confounding</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Lab 6: observational logs built from an RCT, then an agent's analysis audited</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>PROPOSAL PRESENTATIONS. Lab 7 (optional, ungraded, take-home): observational methods on logs built from an RCT, then an agent's analysis audited</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="n"/>
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>Instrumental variables</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="I10" s="8" t="inlineStr">
         <is>
           <t>H4 Instrumental variables</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Thu 12 Nov</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>DML I. The partially linear model; residualisation (FWL) and what theta averages when effects vary; why plug-in ML fails (regularisation and overfitting bias); cross-fitting; orthogonality in words; price elasticity</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>DML II. Inference and repeated splits; choice of nuisance learners; overlap with a continuous treatment; the interactive model and AIPW scores; DML for CATE; omitted-variable sensitivity bounds and benchmarking</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>PROPOSAL PRESENTATIONS</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>Lab 7 (DML, take-home); A3</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>A2 (Sun)</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Lab 8: DML on scanner data (in class)</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>A2 (Sun 15 Nov)</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Regression discontinuity</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>H5 Regression discontinuity</t>
         </is>
@@ -842,31 +906,32 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
+          <t>Tue 17 Nov</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
           <t>GenAI I: simulators. From standardisation to a learned simulator; planting effects and confounding; estimator testbed vs pipeline testbed (regret vs oracle); backtests, support, compounding error, home advantage; planted vs asserted truth (silicon samples, CEVAE)</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>GenAI II: features. LLMs as measurement instruments; labels by role (outcome, control, modifier, treatment) and bias direction; gold subsamples with PPI and DSL; embeddings as DML controls; leakage and overlap collapse</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Lab 8: LLM labels and embeddings as causal variables</t>
-        </is>
-      </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>Lab 9: LLM labels and embeddings as causal variables</t>
         </is>
       </c>
       <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>Causal transformer</t>
         </is>
       </c>
-      <c r="H12" s="4" t="n"/>
+      <c r="I12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
@@ -874,31 +939,40 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
+          <t>Thu 19 Nov</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
           <t>Panel data I: basics. Adoption-date potential outcomes and the ATT; before-after and its failures (trends, seasonality, regression to the mean); comparisons across units; unit and time fixed effects; the within transformation; what fixed effects cannot remove</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Panel data II: DiD. Parallel trends and no anticipation; 2x2 DiD and the ATT; parallel trends in levels vs logs; TWFE with one adoption date; event studies; pre-trend tests and their limits; trend sensitivity (breakdown drift); inference with one change per unit and clustered SEs; a warning on staggered timing</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Lab 9: evaluating an AI rollout with DiD</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="n"/>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Lab 10: evaluating an AI rollout with DiD</t>
+        </is>
+      </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>A3 (Fri); revised identification plan (Sat)</t>
+          <t>A4</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
+          <t>A3 (Fri 20 Nov); revised identification plan (Sat 21 Nov)</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
           <t>Staggered DiD</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>H6 Staggered adoption</t>
         </is>
@@ -910,56 +984,84 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
+          <t>Tue 24 Nov</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
           <t>EXAM II (M5 to M10)</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Panel data III: synthetic controls. One treated unit; donor weights and pre-period fit; interpolation vs extrapolation; the factor-model rationale and a long pre-period; design before the post-period; placebo inference in space and in time, and when a rank is a p-value; leave-one-out; limits (extreme units, spillovers, anticipation, local shocks); SC vs DiD</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Lab 10: synthetic control from scratch</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="n"/>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>A4 (Sun)</t>
-        </is>
-      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Lab 11: synthetic control from scratch</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="n"/>
       <c r="G14" s="8" t="inlineStr">
         <is>
+          <t>A4 (Sun 29 Nov)</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
           <t>Synthetic DiD; matrix completion</t>
         </is>
       </c>
-      <c r="H14" s="8" t="n"/>
+      <c r="I14" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="9" t="n"/>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Thu 26 Nov</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>NO MEETING (Thanksgiving)</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
+      <c r="H15" s="11" t="n"/>
+      <c r="I15" s="11" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Tue 1 Dec</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>FINAL PRESENTATIONS</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr"/>
-      <c r="D15" s="8" t="inlineStr"/>
-      <c r="E15" s="8" t="n"/>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Final slides (the Wednesday before); final report (the following Thursday)</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr"/>
-      <c r="H15" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Final slides, abstract and report (Tue 8 Dec)</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="n"/>
+      <c r="I16" s="8" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F15"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -984,7 +1086,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI labs cover the four roles: tool (Lab 1), decision-maker (Lab 4), source of data (Lab 8), intervention (Lab 9). Lab 6 adds an agent as analyst.</t>
+          <t>Labs 1 to 11 go with Meetings 1 to 11. Ten are graded, 1 point each; Lab 7 is optional and ungraded (its methods are graded in A3). Notebooks are expected soon after their meeting. AI roles: tool (Lab 2), decision-maker (Lab 5), analyst (Lab 7, optional), source of data (Lab 9), intervention (Lab 10).</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1120,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -1038,14 +1140,14 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Refresh pandas and numpy; conditional means; LLN, CLT and standard errors by simulation; bootstrap; confirm OLS on a dummy equals the difference in means. Finish by building a potential-outcomes simulator that verifies naive = ATT + selection bias. Ungraded</t>
+          <t>Refresh pandas and numpy; conditional means; LLN, CLT and standard errors by simulation; bootstrap; confirm OLS on a dummy equals the difference in means. Finish by building a potential-outcomes simulator that verifies naive = ATT + selection bias</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -1072,7 +1174,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1099,7 +1201,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -1126,7 +1228,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -1146,14 +1248,14 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Evaluate four top-20% rules by IPW with the known propensity: random, a response model, a causal forest, and an LLM reading profiles under two prompts ("likely to buy" vs "the coupon changes the purchase"). Qini curves and RATE for the model rules; bootstrap intervals</t>
+          <t>Evaluate four top-20% rules by IPW with the known propensity: random, a response model, a causal forest, and an LLM reading profiles under two prompts ("likely to buy" vs "the coupon changes the purchase"). Qini curves and RATE for the model rules; bootstrap intervals. Recalibrate the forest's score by isotonic regression; freeze each list on a selection fold, then evaluate on a separate fold; compare two lists with a paired SE</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -1173,19 +1275,19 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Greedy and LP allocation under a budget and contact caps; read off the shadow price; compare allocation on point estimates vs lower bounds; fit a depth-2 policy tree on DR scores; compare everything on held-out policy value</t>
+          <t>Greedy and LP allocation under a budget and contact caps; read off the shadow price; compare allocation on point estimates vs lower bounds; fit a depth-2 policy tree on DR scores; compare everything on held-out policy value. Optional: a group constraint and its price</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Semi-synthetic; agentic lab</t>
+          <t>Semi-synthetic; optional and ungraded (take-home)</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1200,19 +1302,19 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>(1) Draw the DAG and pick the adjustment set; compare naive, regression, IPW, AIPW and matching estimates with the RCT truth; overlap and trimming. (2) Run a provided tool-calling agent on the same logs, audit its controls and estimate, then add one guardrail (reject post-treatment controls) and rerun</t>
+          <t>(1) Observational methods: draw the DAG and pick the adjustment set; compare naive, regression, IPW, AIPW and matching estimates with the RCT truth; overlap and trimming. (2) Shorter: run a provided tool-calling agent on the same logs, audit its controls and estimate, then add one guardrail (reject post-treatment controls) and rerun. The methods in part 1 are graded in A3</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Real data; from scratch (take-home)</t>
+          <t>Real data; from scratch (in class)</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1234,7 +1336,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -1261,7 +1363,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -1288,7 +1390,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1378,12 +1480,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>After M2</t>
+          <t>Thu 22 Oct (M2)</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Fri W2</t>
+          <t>Fri 30 Oct</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -1410,12 +1512,12 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>After M5</t>
+          <t>Tue 3 Nov (M5)</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Sun W4</t>
+          <t>Sun 15 Nov</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -1442,59 +1544,59 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>After M8</t>
+          <t>Tue 10 Nov (M7)</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Fri W5</t>
+          <t>Fri 20 Nov</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>M6 to M8</t>
+          <t>M7 to M9</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>The same decision, from observational logs only: DAG and adjustment set; ATE and CATE by regression, AIPW and DML; overlap and trimming. The submitted policy is scored on the locked RCT set next to an RCT-trained benchmark. Sensitivity: how strong hidden confounding must be to change the chosen policy</t>
+          <t>The same decision, from observational logs only. (1) DAG and adjustment set; regression, IPW and AIPW estimates; overlap and trimming (the methods of Lab 7). (2) DML on the same logs, compared with (1) and with the locked RCT. (3) Generative AI for evaluation: a simulator fitted to the coupon logs, with a planted effect and a dial for hidden confounding, as a testbed for each estimator's bias and coverage and for whether the policy ranking holds as confounding grows. An LLM-coded feature is to be decided (depends on the problem and data). The submitted policy is scored on the locked RCT set next to an RCT-trained benchmark. Memo with a sensitivity bound: how strong hidden confounding must be to change the chosen policy</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Allowed, disclosed</t>
+          <t>Allowed, disclosed; simulator as testbed</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>A4: Stress-test the pricing pipeline</t>
+          <t>A4: Did the AI assistant pay?</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>After M9</t>
+          <t>Thu 19 Nov (M10)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Sun W6</t>
+          <t>Sun 29 Nov</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>M8 to M9</t>
+          <t>M10 to M11</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Two pretrained hotel-demand simulators (neural vs boosted outcome models), each with a dial for hidden confounding. Run predict-then-optimize, DML-then-optimize and one pipeline of your choice; measure revenue regret against the oracle across confounding levels; check whether the ranking holds across simulators and outside the logged price range. Recommend a pipeline and a deployment check (holdout or switchback)</t>
+          <t>Panel data. Evaluate the rollout of an AI store assistant: before-after, 2x2 DiD and TWFE with store and period effects; an event study; what the pre-period can and cannot rule out (breakdown drift); store-clustered SEs; why staggered timing needs a different design. Then a synthetic control for one flagship store, with placebos and leave-one-out, and a comparison with DiD. Decision memo in margin, not sales</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Simulator as testbed; tools allowed</t>
+          <t>Allowed, disclosed</t>
         </is>
       </c>
     </row>
@@ -1513,16 +1615,16 @@
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Checked: one major deliverable per week; at most two graded deadlines in any 72 hours; nothing due on an exam day or the weekend before one. Tuesday labs due Thursday; Thursday labs due the following Monday (exceptions: Lab 3 Wed, Lab 10 Sat).</t>
+          <t>Checked: one major deliverable per week; at most two graded deadlines in any 72 hours; nothing due on an exam day or the weekend before one. Lab notebooks are expected soon after their meeting and carry no fixed deadline. No meeting on Thu 26 Nov (Thanksgiving).</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1636,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Graded (labs, exams)</t>
+          <t>Exams and presentations</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1551,138 +1653,126 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Lab 0 (ungraded)</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr"/>
+          <t>1 (20-22 Oct)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Project pairs (Thu 22 Oct)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Lab 1 (Mon), Lab 2 (Thu)</t>
-        </is>
-      </c>
+          <t>2 (27-29 Oct)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>A1 (Fri)</t>
+          <t>A1 (Fri 30 Oct)</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Question and data idea (Thu)</t>
+          <t>Question and data idea (Thu 29 Oct)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3 (3-5 Nov)</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Exam I (Tue), Lab 3 (Wed), Lab 4 (Thu)</t>
+          <t>Exam I (Tue 3 Nov)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Proposal (Sun)</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr"/>
+          <t>Proposal (Sun 8 Nov)</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>4 (10-12 Nov)</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Lab 5 (Mon), Lab 6 (Thu)</t>
+          <t>Proposal presentations (Tue 10 Nov)</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>A2 (Sun)</t>
+          <t>A2 (Sun 15 Nov)</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Proposal presentations (Thu)</t>
+          <t>Lab 7 (optional)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Lab 7 (Mon), Lab 8 (Thu)</t>
-        </is>
-      </c>
+          <t>5 (17-19 Nov)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n"/>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>A3 (Fri)</t>
+          <t>A3 (Fri 20 Nov)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Revised identification plan (Sat)</t>
+          <t>Revised identification plan (Sat 21 Nov)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>6 (24 Nov)</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Lab 9 (Mon), Exam II (Thu), Lab 10 (Sat)</t>
+          <t>Exam II (Tue 24 Nov); no meeting Thu 26 Nov (Thanksgiving)</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>A4 (Sun)</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr"/>
+          <t>A4 (Sun 29 Nov)</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>7 (1 Dec)</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Presentations (Thu)</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Final slides (Wed)</t>
-        </is>
-      </c>
+          <t>Final presentations (Tue 1 Dec)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n"/>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Draft to peer pair (Sat)</t>
+          <t>Draft report to peer pair (Thu 3 Dec); peer review returned (Sun 6 Dec)</t>
         </is>
       </c>
     </row>
@@ -1692,17 +1782,13 @@
           <t>8</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr"/>
+      <c r="B11" s="6" t="n"/>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Final report (Thu)</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Peer review returned (Mon)</t>
-        </is>
-      </c>
+          <t>Final slides, abstract and report (Tue 8 Dec)</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:D11"/>
@@ -2032,7 +2118,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Staggered DiD stays in bonus reading, but Panel II gets a warning slide and Lab 9 an optional extension.</t>
+          <t>Staggered DiD stays in bonus reading. Decided (8 Oct): Panel II has a warning slide (M10 deck); Lab 10 has an optional extension.</t>
         </is>
       </c>
     </row>
@@ -2095,12 +2181,12 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>No panel assignment</t>
+          <t>A4 is a panel assignment</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>DiD examined on Exam II and practised in Labs 9 and 10 and final projects. Alternative: make A4 a DiD evaluation of the AI rollout and fold the simulator into Lab 8.</t>
+          <t>Decided (9 Oct): A4 evaluates the AI-assistant rollout with DiD and the flagship with synthetic control (M10 to M11). The hotel-simulator pipeline assignment is retired; generative AI as an evaluation testbed moves into A3.</t>
         </is>
       </c>
     </row>
@@ -2134,7 +2220,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Lab 8 (cached LLM outputs, gold labels) and A4 (two simulators with a confounding dial) need the most up-front work.</t>
+          <t>Lab 9 (cached LLM outputs, gold labels) and the A3 simulator of the coupon logs (built on the generator behind Lab 7) need the most up-front work.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Spelling pass: US spelling in all student-facing files, case files and the schedule
Mechanical conversion under editorial-guide Section 3 (spelling pass, part 1):
-ise/-isation to -ize/-ization, -our to -or, -tre to -ter, single l (modeled,
labeled), program, judgment, defense, license, analog, catalog, gray,
artifact, toward. 553 lines in 36 files plus 11 schedule cells. Labels,
references, file names, URLs, code and reading-list titles untouched. Curly
quotes in the Markdown cases straightened. slides08_check.py follows the new
spelling of the Case B key sentence it verifies.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DLgfSPmYNxNjqrXY4qwk61
</commit_message>
<xml_diff>
--- a/plan/schedule.xlsx
+++ b/plan/schedule.xlsx
@@ -600,7 +600,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Causal basics II: causal graphs. DAGs as assumptions; forks, chains, colliders; backdoor paths; randomisation as graph surgery; Simpson's paradox; identification vs estimation vs inference</t>
+          <t>Causal basics II: causal graphs. DAGs as assumptions; forks, chains, colliders; backdoor paths; randomization as graph surgery; Simpson's paradox; identification vs estimation vs inference</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -628,12 +628,12 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Experiments I: estimation. Analyse as drawn (the ITT); sample-ratio checks; Fisher's test and Neyman's variance; the usual SE is conservative; difference in means as OLS on a dummy with robust SEs; testing against the break-even, and an interval on net value; transport to a new campaign</t>
+          <t>Experiments I: estimation. Analyze as drawn (the ITT); sample-ratio checks; Fisher's test and Neyman's variance; the usual SE is conservative; difference in means as OLS on a dummy with robust SEs; testing against the break-even, and an interval on net value; transport to a new campaign</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Experiments II: design. Fixing the plan in writing; power and MDE for a decision; CUPED; randomisation unit, interference and clustered SEs; peeking and multiple metrics; to close, noncompliance in an RCT: ITT and first stage, compliance types, the LATE (potential outcomes; the draw as the instrument)</t>
+          <t>Experiments II: design. Fixing the plan in writing; power and MDE for a decision; CUPED; randomization unit, interference and clustered SEs; peeking and multiple metrics; to close, noncompliance in an RCT: ITT and first stage, compliance types, the LATE (potential outcomes; the draw as the instrument)</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>CATE IV: causal forests. Forests as adaptive neighbours; the forest estimate and local centering (link to the R-learner); CATE intervals and their limits; variable-importance pitfalls; BLP calibration test and GATES</t>
+          <t>CATE IV: causal forests. Forests as adaptive neighbors; the forest estimate and local centering (link to the R-learner); CATE intervals and their limits; variable-importance pitfalls; BLP calibration test and GATES</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>Evaluating prioritisation rules</t>
+          <t>Evaluating prioritization rules</t>
         </is>
       </c>
       <c r="I8" s="8" t="n"/>
@@ -797,7 +797,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>CATE VII: policy learning. Predict-then-optimise, decision-focused learning and policy learning as one spectrum; empirical welfare maximisation with DR scores; policy learning as weighted classification; policy trees; regret and policy-class complexity; deploying with holdouts; bandits as continuous experimentation; what the sum assumes (interference, support)</t>
+          <t>CATE VII: policy learning. Predict-then-optimize, decision-focused learning and policy learning as one spectrum; empirical welfare maximization with DR scores; policy learning as weighted classification; policy trees; regret and policy-class complexity; deploying with holdouts; bandits as continuous experimentation; what the sum assumes (interference, support)</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Observational data I: identification and adjustment. Logs produced by a targeting rule; exchangeability, overlap, consistency; standardisation (g-computation) and IPW; the balancing property; what regression adjustment estimates; good and bad controls (mediators, colliders, M-bias, post-treatment variables)</t>
+          <t>Observational data I: identification and adjustment. Logs produced by a targeting rule; exchangeability, overlap, consistency; standardization (g-computation) and IPW; the balancing property; what regression adjustment estimates; good and bad controls (mediators, colliders, M-bias, post-treatment variables)</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>DML I. The partially linear model; residualisation (FWL) and what theta averages when effects vary; why plug-in ML fails (regularisation and overfitting bias); cross-fitting; orthogonality in words; price elasticity</t>
+          <t>DML I. The partially linear model; residualization (FWL) and what theta averages when effects vary; why plug-in ML fails (regularization and overfitting bias); cross-fitting; orthogonality in words; price elasticity</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>GenAI I: simulators. From standardisation to a learned simulator; planting effects and confounding; estimator testbed vs pipeline testbed (regret vs oracle); backtests, support, compounding error, home advantage; planted vs asserted truth (silicon samples, CEVAE)</t>
+          <t>GenAI I: simulators. From standardization to a learned simulator; planting effects and confounding; estimator testbed vs pipeline testbed (regret vs oracle); backtests, support, compounding error, home advantage; planted vs asserted truth (silicon samples, CEVAE)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1090,6 +1090,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1260,7 +1261,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>From scratch (optimisation); real data</t>
+          <t>From scratch (optimization); real data</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1628,6 +1629,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1820,6 +1822,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1913,7 +1916,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Evaluating prioritisation rules</t>
+          <t>Evaluating prioritization rules</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -2071,6 +2074,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>

</xml_diff>